<commit_message>
Remove obsolete code and streamline remaining files
</commit_message>
<xml_diff>
--- a/BlueBridge_TOFU_BizDev_V1.xlsx
+++ b/BlueBridge_TOFU_BizDev_V1.xlsx
@@ -494,7 +494,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
@@ -647,7 +647,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>0 RSS items; 0 discovery hits; 0 trigger events; errors: MedTech AI Funding: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | SaMD Series A: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | medical device: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | FDA clearance AI: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | digital health regulatory clearance: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt;</t>
+          <t>0 RSS items; 0 discovery hits; 0 trigger events; errors: MedTech AI Funding: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | SaMD Series A: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | medical device: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | FDA clearance AI: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | digital health regulatory clearance: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Trinity College Dublin" spinout medical device: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Trinity College Dublin" spinout digital health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Trinity College Dublin" spinout medtech: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Trinity College Dublin" spinout diagnostics: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Trinity College Dublin" "campus company" health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Trinity College Dublin" startup healthcare: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Trinity College Dublin" startup "medical device": &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Trinity College Dublin" commercialisation health startup: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "RCSI" spinout medical device: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "RCSI" spinout digital health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "RCSI" spinout medtech: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "RCSI" spinout diagnostics: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "RCSI" "campus company" health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "RCSI" startup healthcare: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "RCSI" startup "medical device": &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "RCSI" commercialisation health startup: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "UCD" spinout medical device: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "UCD" spinout digital health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "UCD" spinout medtech: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "UCD" spinout diagnostics: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "UCD" "campus company" health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "UCD" startup healthcare: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "UCD" startup "medical device": &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "UCD" commercialisation health startup: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Galway" spinout medical device: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Galway" spinout digital health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Galway" spinout medtech: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Galway" spinout diagnostics: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Galway" "campus company" health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Galway" startup healthcare: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Galway" startup "medical device": &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Galway" commercialisation health startup: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Limerick" spinout medical device: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Limerick" spinout digital health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Limerick" spinout medtech: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Limerick" spinout diagnostics: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Limerick" "campus company" health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Limerick" startup healthcare: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Limerick" startup "medical device": &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Limerick" commercialisation health startup: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University College Cork" spinout medical device: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University College Cork" spinout digital health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University College Cork" spinout medtech: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University College Cork" spinout diagnostics: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University College Cork" "campus company" health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University College Cork" startup healthcare: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University College Cork" startup "medical device": &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University College Cork" commercialisation health startup: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Queen's University Belfast" spinout medical device: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Queen's University Belfast" spinout digital health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Queen's University Belfast" spinout medtech: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Queen's University Belfast" spinout diagnostics: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Queen's University Belfast" "campus company" health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Queen's University Belfast" startup healthcare: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Queen's University Belfast" startup "medical device": &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Queen's University Belfast" commercialisation health startup: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Oxford" spinout medical device: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Oxford" spinout digital health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Oxford" spinout medtech: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Oxford" spinout diagnostics: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Oxford" "campus company" health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Oxford" startup healthcare: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Oxford" startup "medical device": &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Oxford" commercialisation health startup: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Cambridge" spinout medical device: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Cambridge" spinout digital health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Cambridge" spinout medtech: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Cambridge" spinout diagnostics: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Cambridge" "campus company" health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Cambridge" startup healthcare: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Cambridge" startup "medical device": &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Cambridge" commercialisation health startup: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Imperial College London" spinout medical device: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Imperial College London" spinout digital health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Imperial College London" spinout medtech: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Imperial College London" spinout diagnostics: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Imperial College London" "campus company" health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Imperial College London" startup healthcare: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Imperial College London" startup "medical device": &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Imperial College London" commercialisation health startup: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "King's College London" spinout medical device: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "King's College London" spinout digital health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "King's College London" spinout medtech: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "King's College London" spinout diagnostics: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "King's College London" "campus company" health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "King's College London" startup healthcare: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "King's College London" startup "medical device": &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "King's College London" commercialisation health startup: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "UCL" spinout medical device: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "UCL" spinout digital health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "UCL" spinout medtech: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "UCL" spinout diagnostics: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "UCL" "campus company" health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "UCL" startup healthcare: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "UCL" startup "medical device": &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "UCL" commercialisation health startup: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Edinburgh" spinout medical device: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Edinburgh" spinout digital health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Edinburgh" spinout medtech: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Edinburgh" spinout diagnostics: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Edinburgh" "campus company" health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Edinburgh" startup healthcare: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Edinburgh" startup "medical device": &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Edinburgh" commercialisation health startup: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Manchester" spinout medical device: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Manchester" spinout digital health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Manchester" spinout medtech: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Manchester" spinout diagnostics: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Manchester" "campus company" health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Manchester" startup healthcare: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Manchester" startup "medical device": &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Manchester" commercialisation health startup: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Leeds" spinout medical device: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Leeds" spinout digital health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Leeds" spinout medtech: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Leeds" spinout diagnostics: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Leeds" "campus company" health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Leeds" startup healthcare: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Leeds" startup "medical device": &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Leeds" commercialisation health startup: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Sheffield" spinout medical device: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Sheffield" spinout digital health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Sheffield" spinout medtech: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Sheffield" spinout diagnostics: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Sheffield" "campus company" health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Sheffield" startup healthcare: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Sheffield" startup "medical device": &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "University of Sheffield" commercialisation health startup: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "ETH Zurich" spinout medical device: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "ETH Zurich" spinout digital health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "ETH Zurich" spinout medtech: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "ETH Zurich" spinout diagnostics: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "ETH Zurich" "campus company" health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "ETH Zurich" startup healthcare: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "ETH Zurich" startup "medical device": &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "ETH Zurich" commercialisation health startup: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "KU Leuven" spinout medical device: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "KU Leuven" spinout digital health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "KU Leuven" spinout medtech: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "KU Leuven" spinout diagnostics: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "KU Leuven" "campus company" health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "KU Leuven" startup healthcare: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "KU Leuven" startup "medical device": &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "KU Leuven" commercialisation health startup: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "EPFL" spinout medical device: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "EPFL" spinout digital health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "EPFL" spinout medtech: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "EPFL" spinout diagnostics: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "EPFL" "campus company" health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "EPFL" startup healthcare: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "EPFL" startup "medical device": &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "EPFL" commercialisation health startup: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Technical University of Denmark" spinout medical device: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Technical University of Denmark" spinout digital health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Technical University of Denmark" spinout medtech: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Technical University of Denmark" spinout diagnostics: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Technical University of Denmark" "campus company" health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Technical University of Denmark" startup healthcare: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Technical University of Denmark" startup "medical device": &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Technical University of Denmark" commercialisation health startup: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "TU Delft" spinout medical device: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "TU Delft" spinout digital health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "TU Delft" spinout medtech: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "TU Delft" spinout diagnostics: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "TU Delft" "campus company" health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "TU Delft" startup healthcare: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "TU Delft" startup "medical device": &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "TU Delft" commercialisation health startup: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Karolinska Institutet" spinout medical device: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Karolinska Institutet" spinout digital health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Karolinska Institutet" spinout medtech: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Karolinska Institutet" spinout diagnostics: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Karolinska Institutet" "campus company" health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Karolinska Institutet" startup healthcare: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Karolinska Institutet" startup "medical device": &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Karolinska Institutet" commercialisation health startup: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Technical University of Munich" spinout medical device: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Technical University of Munich" spinout digital health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Technical University of Munich" spinout medtech: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Technical University of Munich" spinout diagnostics: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Technical University of Munich" "campus company" health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Technical University of Munich" startup healthcare: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Technical University of Munich" startup "medical device": &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Technical University of Munich" commercialisation health startup: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Stanford" spinout medical device: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Stanford" spinout digital health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Stanford" spinout medtech: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Stanford" spinout diagnostics: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Stanford" "campus company" health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Stanford" startup healthcare: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Stanford" startup "medical device": &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "Stanford" commercialisation health startup: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "MIT" spinout medical device: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "MIT" spinout digital health: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "MIT" spinout medtech: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "MIT" spinout diagnostics: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | "MIT" "campus company" health: &lt;urlopen error [WinError</t>
         </is>
       </c>
     </row>
@@ -1835,7 +1835,7 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>3 university spinout pages; 0 discovery hits; 0 trigger events; errors: https://www.tcd.ie/innovation/: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | https://www.tcd.ie/innovation/what-we-do/for-startups-and-spinouts/: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | https://www.tcd.ie/innovation/news-events/: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt;</t>
+          <t>3 university spinout pages; 0 discovery hits; 0 trigger events; errors: https://www.tcd.ie/innovation/: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | https://www.tcd.ie/innovation/what-we-do/for-startups-and-spinouts/: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt; | https://www.tcd.ie/innovation/about/news-and-events/: &lt;urlopen error [WinError 10013] An attempt was made to access a socket in a way forbidden by its access permissions&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>